<commit_message>
ACT-117C: actualizar template con nuevo archivo ACT-117C.xlsx
</commit_message>
<xml_diff>
--- a/Documentos/ACT-117C.xlsx
+++ b/Documentos/ACT-117C.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\M2A (GD)\CARRETERAS\DOCUMENTOS CARRETERAS\FORMAS Y DOCUMENTOS ACT\Formas con celdas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Enrique Saavedra\Documents\PROGRAMAS AI\Programa ACT\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B279836-7F72-4891-A32A-F0FEECB96D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A14CDA-CF04-4CEB-8D5C-DB18B1293F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{94FC3A84-A9BC-4322-B311-2768DE3D711D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{94FC3A84-A9BC-4322-B311-2768DE3D711D}"/>
   </bookViews>
   <sheets>
     <sheet name="MPPR- ACT-117C (p5)" sheetId="1" r:id="rId1"/>
@@ -1031,6 +1031,160 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="8" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="8" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1043,11 +1197,57 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="167" fontId="17" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1061,210 +1261,10 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="15" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1564,6 +1564,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="ValidationLists"/>
       <sheetName val="Document Worksheet"/>
@@ -2207,7 +2210,6 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="MPPR- ACT-117C (p1)"/>
@@ -2750,61 +2752,61 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="146" t="s">
+      <c r="A2" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="146"/>
-      <c r="C2" s="146"/>
-      <c r="D2" s="146"/>
-      <c r="E2" s="146"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="146"/>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
-      <c r="K2" s="146"/>
-      <c r="L2" s="147"/>
-      <c r="M2" s="147"/>
-      <c r="N2" s="147"/>
-      <c r="O2" s="147"/>
-      <c r="P2" s="147"/>
-      <c r="Q2" s="147"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="83"/>
+      <c r="M2" s="83"/>
+      <c r="N2" s="83"/>
+      <c r="O2" s="83"/>
+      <c r="P2" s="83"/>
+      <c r="Q2" s="83"/>
     </row>
     <row r="3" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="148" t="s">
+      <c r="A3" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="148"/>
-      <c r="C3" s="148"/>
-      <c r="D3" s="148"/>
-      <c r="E3" s="148"/>
-      <c r="F3" s="148"/>
-      <c r="G3" s="148"/>
-      <c r="H3" s="148"/>
-      <c r="I3" s="148"/>
-      <c r="J3" s="148"/>
-      <c r="K3" s="148"/>
-      <c r="L3" s="147"/>
-      <c r="M3" s="147"/>
-      <c r="N3" s="147"/>
-      <c r="O3" s="147"/>
-      <c r="P3" s="147"/>
-      <c r="Q3" s="147"/>
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="84"/>
+      <c r="I3" s="84"/>
+      <c r="J3" s="84"/>
+      <c r="K3" s="84"/>
+      <c r="L3" s="83"/>
+      <c r="M3" s="83"/>
+      <c r="N3" s="83"/>
+      <c r="O3" s="83"/>
+      <c r="P3" s="83"/>
+      <c r="Q3" s="83"/>
     </row>
     <row r="4" spans="1:17" ht="18" x14ac:dyDescent="0.35">
-      <c r="A4" s="149" t="s">
+      <c r="A4" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="149"/>
-      <c r="C4" s="149"/>
-      <c r="D4" s="149"/>
-      <c r="E4" s="149"/>
-      <c r="F4" s="149"/>
-      <c r="G4" s="149"/>
-      <c r="H4" s="149"/>
-      <c r="I4" s="149"/>
-      <c r="J4" s="149"/>
-      <c r="K4" s="149"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="85"/>
+      <c r="H4" s="85"/>
+      <c r="I4" s="85"/>
+      <c r="J4" s="85"/>
+      <c r="K4" s="85"/>
     </row>
     <row r="5" spans="1:17" ht="11.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
@@ -2820,37 +2822,37 @@
       <c r="K5" s="1"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="150" t="s">
+      <c r="A6" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="150"/>
-      <c r="C6" s="150"/>
-      <c r="D6" s="150"/>
-      <c r="E6" s="150"/>
-      <c r="F6" s="150"/>
-      <c r="G6" s="150"/>
-      <c r="H6" s="150"/>
-      <c r="I6" s="150"/>
-      <c r="J6" s="150"/>
-      <c r="K6" s="150"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="86"/>
+      <c r="D6" s="86"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="86"/>
+      <c r="G6" s="86"/>
+      <c r="H6" s="86"/>
+      <c r="I6" s="86"/>
+      <c r="J6" s="86"/>
+      <c r="K6" s="86"/>
     </row>
     <row r="7" spans="1:17" ht="29.7" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="151" t="s">
+      <c r="C7" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="151"/>
-      <c r="E7" s="151"/>
-      <c r="F7" s="151"/>
+      <c r="D7" s="80"/>
+      <c r="E7" s="80"/>
+      <c r="F7" s="80"/>
       <c r="H7" t="s">
         <v>6</v>
       </c>
-      <c r="J7" s="141">
+      <c r="J7" s="81">
         <v>44986</v>
       </c>
-      <c r="K7" s="141"/>
+      <c r="K7" s="81"/>
     </row>
     <row r="8" spans="1:17" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -2865,118 +2867,118 @@
       <c r="H8" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="143">
+      <c r="J8" s="87">
         <v>8</v>
       </c>
-      <c r="K8" s="143"/>
+      <c r="K8" s="87"/>
       <c r="P8" s="4"/>
     </row>
     <row r="9" spans="1:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="138" t="s">
+      <c r="C9" s="88" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="138"/>
-      <c r="E9" s="138"/>
-      <c r="F9" s="138"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
       <c r="H9" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="144">
+      <c r="J9" s="89">
         <v>44977</v>
       </c>
-      <c r="K9" s="143"/>
-      <c r="P9" s="145"/>
-      <c r="Q9" s="145"/>
+      <c r="K9" s="87"/>
+      <c r="P9" s="90"/>
+      <c r="Q9" s="90"/>
     </row>
     <row r="10" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="138" t="s">
+      <c r="C10" s="88" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="138"/>
+      <c r="D10" s="88"/>
       <c r="E10" s="5"/>
       <c r="G10" s="6" t="s">
         <v>15</v>
       </c>
       <c r="H10" s="6"/>
-      <c r="J10" s="141">
+      <c r="J10" s="81">
         <v>44348</v>
       </c>
-      <c r="K10" s="141"/>
+      <c r="K10" s="81"/>
     </row>
     <row r="11" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="138" t="s">
+      <c r="C11" s="88" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="138"/>
+      <c r="D11" s="88"/>
       <c r="G11" s="6" t="s">
         <v>18</v>
       </c>
       <c r="H11" s="6"/>
-      <c r="J11" s="141">
+      <c r="J11" s="81">
         <v>44767</v>
       </c>
-      <c r="K11" s="141"/>
+      <c r="K11" s="81"/>
     </row>
     <row r="12" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="138" t="s">
+      <c r="C12" s="88" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="138"/>
+      <c r="D12" s="88"/>
       <c r="G12" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H12" s="6"/>
-      <c r="J12" s="142">
+      <c r="J12" s="91">
         <v>44812</v>
       </c>
-      <c r="K12" s="141"/>
+      <c r="K12" s="81"/>
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="138" t="s">
+      <c r="C13" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="138"/>
+      <c r="D13" s="88"/>
       <c r="G13" s="6" t="s">
         <v>24</v>
       </c>
       <c r="H13" s="6"/>
-      <c r="J13" s="139">
+      <c r="J13" s="92">
         <v>3137499</v>
       </c>
-      <c r="K13" s="139"/>
+      <c r="K13" s="92"/>
     </row>
     <row r="14" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="138" t="s">
+      <c r="C14" s="88" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="138"/>
+      <c r="D14" s="88"/>
       <c r="G14" s="6" t="s">
         <v>27</v>
       </c>
       <c r="H14" s="6"/>
-      <c r="J14" s="139">
+      <c r="J14" s="92">
         <v>4027901</v>
       </c>
-      <c r="K14" s="139"/>
+      <c r="K14" s="92"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H15" s="8"/>
@@ -3025,11 +3027,11 @@
       <c r="D18" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="140" t="s">
+      <c r="E18" s="94" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="140"/>
-      <c r="G18" s="140"/>
+      <c r="F18" s="94"/>
+      <c r="G18" s="94"/>
       <c r="H18" s="10" t="s">
         <v>33</v>
       </c>
@@ -3108,11 +3110,11 @@
         <v>43</v>
       </c>
       <c r="D21" s="11"/>
-      <c r="E21" s="125" t="s">
+      <c r="E21" s="95" t="s">
         <v>44</v>
       </c>
-      <c r="F21" s="126"/>
-      <c r="G21" s="127"/>
+      <c r="F21" s="96"/>
+      <c r="G21" s="97"/>
       <c r="H21" s="11" t="s">
         <v>39</v>
       </c>
@@ -3136,11 +3138,11 @@
         <v>45</v>
       </c>
       <c r="D22" s="11"/>
-      <c r="E22" s="125" t="s">
+      <c r="E22" s="95" t="s">
         <v>46</v>
       </c>
-      <c r="F22" s="126"/>
-      <c r="G22" s="127"/>
+      <c r="F22" s="96"/>
+      <c r="G22" s="97"/>
       <c r="H22" s="11" t="s">
         <v>39</v>
       </c>
@@ -3165,11 +3167,11 @@
         <v>47</v>
       </c>
       <c r="D23" s="11"/>
-      <c r="E23" s="125" t="s">
+      <c r="E23" s="95" t="s">
         <v>48</v>
       </c>
-      <c r="F23" s="126"/>
-      <c r="G23" s="127"/>
+      <c r="F23" s="96"/>
+      <c r="G23" s="97"/>
       <c r="H23" s="11" t="s">
         <v>39</v>
       </c>
@@ -3194,11 +3196,11 @@
         <v>49</v>
       </c>
       <c r="D24" s="11"/>
-      <c r="E24" s="122" t="s">
+      <c r="E24" s="98" t="s">
         <v>50</v>
       </c>
-      <c r="F24" s="123"/>
-      <c r="G24" s="124"/>
+      <c r="F24" s="99"/>
+      <c r="G24" s="100"/>
       <c r="H24" s="11" t="s">
         <v>51</v>
       </c>
@@ -3222,11 +3224,11 @@
         <v>52</v>
       </c>
       <c r="D25" s="11"/>
-      <c r="E25" s="122" t="s">
+      <c r="E25" s="98" t="s">
         <v>53</v>
       </c>
-      <c r="F25" s="123"/>
-      <c r="G25" s="124"/>
+      <c r="F25" s="99"/>
+      <c r="G25" s="100"/>
       <c r="H25" s="11" t="s">
         <v>39</v>
       </c>
@@ -3250,11 +3252,11 @@
         <v>54</v>
       </c>
       <c r="D26" s="11"/>
-      <c r="E26" s="122" t="s">
+      <c r="E26" s="98" t="s">
         <v>55</v>
       </c>
-      <c r="F26" s="123"/>
-      <c r="G26" s="124"/>
+      <c r="F26" s="99"/>
+      <c r="G26" s="100"/>
       <c r="H26" s="11" t="s">
         <v>39</v>
       </c>
@@ -3278,11 +3280,11 @@
         <v>56</v>
       </c>
       <c r="D27" s="11"/>
-      <c r="E27" s="125" t="s">
+      <c r="E27" s="95" t="s">
         <v>57</v>
       </c>
-      <c r="F27" s="126"/>
-      <c r="G27" s="127"/>
+      <c r="F27" s="96"/>
+      <c r="G27" s="97"/>
       <c r="H27" s="11" t="s">
         <v>58</v>
       </c>
@@ -3311,55 +3313,55 @@
       <c r="K28" s="19"/>
     </row>
     <row r="29" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="128" t="s">
+      <c r="A29" s="101" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="129"/>
-      <c r="C29" s="129"/>
-      <c r="D29" s="129"/>
-      <c r="E29" s="129"/>
-      <c r="F29" s="129"/>
-      <c r="G29" s="129"/>
-      <c r="H29" s="129"/>
-      <c r="I29" s="129"/>
-      <c r="J29" s="129"/>
-      <c r="K29" s="130"/>
+      <c r="B29" s="102"/>
+      <c r="C29" s="102"/>
+      <c r="D29" s="102"/>
+      <c r="E29" s="102"/>
+      <c r="F29" s="102"/>
+      <c r="G29" s="102"/>
+      <c r="H29" s="102"/>
+      <c r="I29" s="102"/>
+      <c r="J29" s="102"/>
+      <c r="K29" s="103"/>
       <c r="M29" s="24"/>
     </row>
     <row r="30" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="131"/>
-      <c r="B30" s="132"/>
-      <c r="C30" s="132"/>
-      <c r="D30" s="132"/>
-      <c r="E30" s="132"/>
-      <c r="F30" s="132"/>
-      <c r="G30" s="132"/>
-      <c r="H30" s="132"/>
-      <c r="I30" s="132"/>
-      <c r="J30" s="132"/>
-      <c r="K30" s="133"/>
+      <c r="A30" s="104"/>
+      <c r="B30" s="105"/>
+      <c r="C30" s="105"/>
+      <c r="D30" s="105"/>
+      <c r="E30" s="105"/>
+      <c r="F30" s="105"/>
+      <c r="G30" s="105"/>
+      <c r="H30" s="105"/>
+      <c r="I30" s="105"/>
+      <c r="J30" s="105"/>
+      <c r="K30" s="106"/>
     </row>
     <row r="31" spans="1:13" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="134"/>
-      <c r="B31" s="135"/>
-      <c r="C31" s="135"/>
-      <c r="D31" s="135"/>
-      <c r="E31" s="135"/>
-      <c r="F31" s="135"/>
-      <c r="G31" s="135"/>
-      <c r="H31" s="135"/>
-      <c r="I31" s="135"/>
-      <c r="J31" s="135"/>
-      <c r="K31" s="136"/>
+      <c r="A31" s="107"/>
+      <c r="B31" s="108"/>
+      <c r="C31" s="108"/>
+      <c r="D31" s="108"/>
+      <c r="E31" s="108"/>
+      <c r="F31" s="108"/>
+      <c r="G31" s="108"/>
+      <c r="H31" s="108"/>
+      <c r="I31" s="108"/>
+      <c r="J31" s="108"/>
+      <c r="K31" s="109"/>
     </row>
     <row r="32" spans="1:13" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="28"/>
       <c r="C32" s="9"/>
       <c r="D32" s="28"/>
-      <c r="E32" s="137" t="s">
+      <c r="E32" s="93" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="137"/>
+      <c r="F32" s="93"/>
       <c r="G32" s="29"/>
       <c r="H32" s="28"/>
       <c r="I32" s="7"/>
@@ -3386,12 +3388,12 @@
         <v>62</v>
       </c>
       <c r="B34" s="32"/>
-      <c r="D34" s="118" t="s">
+      <c r="D34" s="110" t="s">
         <v>63</v>
       </c>
-      <c r="E34" s="118"/>
-      <c r="F34" s="118"/>
-      <c r="G34" s="118"/>
+      <c r="E34" s="110"/>
+      <c r="F34" s="110"/>
+      <c r="G34" s="110"/>
       <c r="I34" s="33" t="s">
         <v>64</v>
       </c>
@@ -3423,10 +3425,10 @@
         <v>68</v>
       </c>
       <c r="B36" s="32"/>
-      <c r="D36" s="118" t="s">
+      <c r="D36" s="110" t="s">
         <v>69</v>
       </c>
-      <c r="E36" s="118"/>
+      <c r="E36" s="110"/>
       <c r="F36" s="38"/>
       <c r="G36" s="39"/>
       <c r="I36" s="33" t="s">
@@ -3461,8 +3463,8 @@
       </c>
       <c r="B38" s="32"/>
       <c r="C38" s="33"/>
-      <c r="D38" s="119"/>
-      <c r="E38" s="119"/>
+      <c r="D38" s="111"/>
+      <c r="E38" s="111"/>
       <c r="F38" s="42"/>
       <c r="G38" s="42"/>
       <c r="I38" s="33" t="s">
@@ -3474,14 +3476,14 @@
       <c r="A39" s="32"/>
       <c r="B39" s="32"/>
       <c r="C39" s="33"/>
-      <c r="D39" s="120" t="s">
+      <c r="D39" s="112" t="s">
         <v>75</v>
       </c>
-      <c r="E39" s="120"/>
-      <c r="F39" s="121" t="s">
+      <c r="E39" s="112"/>
+      <c r="F39" s="113" t="s">
         <v>76</v>
       </c>
-      <c r="G39" s="121"/>
+      <c r="G39" s="113"/>
       <c r="I39" s="33" t="s">
         <v>77</v>
       </c>
@@ -3495,10 +3497,10 @@
       </c>
       <c r="B40" s="32"/>
       <c r="C40" s="33"/>
-      <c r="D40" s="118" t="s">
+      <c r="D40" s="110" t="s">
         <v>79</v>
       </c>
-      <c r="E40" s="118"/>
+      <c r="E40" s="110"/>
       <c r="F40" s="38"/>
       <c r="G40" s="43"/>
       <c r="I40" s="33" t="s">
@@ -3516,10 +3518,10 @@
         <v>81</v>
       </c>
       <c r="E41" s="7"/>
-      <c r="F41" s="121" t="s">
+      <c r="F41" s="113" t="s">
         <v>66</v>
       </c>
-      <c r="G41" s="121"/>
+      <c r="G41" s="113"/>
       <c r="I41" s="33" t="s">
         <v>82</v>
       </c>
@@ -3533,10 +3535,10 @@
       </c>
       <c r="B42" s="32"/>
       <c r="C42" s="33"/>
-      <c r="D42" s="118" t="s">
+      <c r="D42" s="110" t="s">
         <v>84</v>
       </c>
-      <c r="E42" s="118"/>
+      <c r="E42" s="110"/>
       <c r="F42" s="38"/>
       <c r="G42" s="43"/>
       <c r="I42" s="33" t="s">
@@ -3572,10 +3574,10 @@
       </c>
       <c r="B45" s="32"/>
       <c r="C45" s="33"/>
-      <c r="D45" s="118" t="s">
+      <c r="D45" s="110" t="s">
         <v>89</v>
       </c>
-      <c r="E45" s="118"/>
+      <c r="E45" s="110"/>
       <c r="F45" s="38"/>
       <c r="G45" s="43"/>
       <c r="I45" s="33" t="s">
@@ -3619,25 +3621,15 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="L2:Q3"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F41:G41"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="J14:K14"/>
@@ -3650,15 +3642,25 @@
     <mergeCell ref="E26:G26"/>
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="A29:K31"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="L2:Q3"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A6:K6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.25" bottom="0.25" header="0.05" footer="0.3"/>
@@ -3755,25 +3757,25 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="47"/>
-      <c r="B4" s="108" t="s">
+      <c r="B4" s="118" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="109"/>
-      <c r="D4" s="109"/>
-      <c r="E4" s="109"/>
-      <c r="F4" s="109"/>
-      <c r="G4" s="109"/>
-      <c r="H4" s="109"/>
-      <c r="I4" s="109"/>
-      <c r="J4" s="109"/>
-      <c r="K4" s="109"/>
-      <c r="L4" s="109"/>
-      <c r="M4" s="109"/>
-      <c r="N4" s="109"/>
-      <c r="O4" s="109"/>
-      <c r="P4" s="109"/>
-      <c r="Q4" s="109"/>
-      <c r="R4" s="110"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="119"/>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119"/>
+      <c r="P4" s="119"/>
+      <c r="Q4" s="119"/>
+      <c r="R4" s="120"/>
       <c r="S4" s="47"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.3">
@@ -3807,17 +3809,17 @@
       <c r="E6" s="47"/>
       <c r="F6" s="47"/>
       <c r="G6" s="47"/>
-      <c r="H6" s="115">
+      <c r="H6" s="121">
         <v>44813</v>
       </c>
-      <c r="I6" s="115"/>
+      <c r="I6" s="121"/>
       <c r="J6" s="50" t="s">
         <v>97</v>
       </c>
-      <c r="K6" s="115">
+      <c r="K6" s="121">
         <v>44977</v>
       </c>
-      <c r="L6" s="115"/>
+      <c r="L6" s="121"/>
       <c r="M6" s="51"/>
       <c r="N6" s="47" t="s">
         <v>98</v>
@@ -3839,15 +3841,15 @@
       <c r="E7" s="47"/>
       <c r="F7" s="47"/>
       <c r="G7" s="47"/>
-      <c r="H7" s="103">
+      <c r="H7" s="122">
         <v>47</v>
       </c>
-      <c r="I7" s="103"/>
+      <c r="I7" s="122"/>
       <c r="J7" s="50"/>
-      <c r="K7" s="103">
+      <c r="K7" s="122">
         <v>48</v>
       </c>
-      <c r="L7" s="103"/>
+      <c r="L7" s="122"/>
       <c r="M7" s="52"/>
       <c r="N7" s="47"/>
       <c r="O7" s="47"/>
@@ -3861,28 +3863,28 @@
       <c r="B8" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="C8" s="116">
+      <c r="C8" s="114">
         <v>164</v>
       </c>
-      <c r="D8" s="116"/>
+      <c r="D8" s="114"/>
       <c r="E8" s="50" t="s">
         <v>100</v>
       </c>
       <c r="F8" s="53">
         <v>2000</v>
       </c>
-      <c r="G8" s="105" t="s">
+      <c r="G8" s="115" t="s">
         <v>101</v>
       </c>
-      <c r="H8" s="105"/>
+      <c r="H8" s="115"/>
       <c r="I8" s="54"/>
       <c r="J8" s="47">
         <v>3</v>
       </c>
-      <c r="K8" s="114" t="s">
+      <c r="K8" s="116" t="s">
         <v>102</v>
       </c>
-      <c r="L8" s="114"/>
+      <c r="L8" s="116"/>
       <c r="M8" s="55"/>
       <c r="N8" s="117">
         <f>C8*F8</f>
@@ -3897,10 +3899,10 @@
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" s="47"/>
       <c r="B9" s="48"/>
-      <c r="C9" s="103">
+      <c r="C9" s="122">
         <v>49</v>
       </c>
-      <c r="D9" s="103"/>
+      <c r="D9" s="122"/>
       <c r="E9" s="47"/>
       <c r="F9" s="56">
         <v>50</v>
@@ -3912,40 +3914,40 @@
       <c r="K9" s="47"/>
       <c r="L9" s="47"/>
       <c r="M9" s="47"/>
-      <c r="N9" s="103">
+      <c r="N9" s="122">
         <v>51</v>
       </c>
-      <c r="O9" s="103"/>
-      <c r="P9" s="103"/>
+      <c r="O9" s="122"/>
+      <c r="P9" s="122"/>
       <c r="Q9" s="47"/>
       <c r="R9" s="49"/>
       <c r="S9" s="47"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" s="47"/>
-      <c r="B10" s="104" t="s">
+      <c r="B10" s="123" t="s">
         <v>103</v>
       </c>
-      <c r="C10" s="105"/>
-      <c r="D10" s="106">
+      <c r="C10" s="115"/>
+      <c r="D10" s="124">
         <v>0</v>
       </c>
-      <c r="E10" s="106"/>
-      <c r="F10" s="112"/>
-      <c r="G10" s="112"/>
-      <c r="H10" s="112"/>
-      <c r="I10" s="112"/>
-      <c r="J10" s="114" t="s">
+      <c r="E10" s="124"/>
+      <c r="F10" s="125"/>
+      <c r="G10" s="125"/>
+      <c r="H10" s="125"/>
+      <c r="I10" s="125"/>
+      <c r="J10" s="116" t="s">
         <v>104</v>
       </c>
-      <c r="K10" s="114"/>
-      <c r="L10" s="114"/>
+      <c r="K10" s="116"/>
+      <c r="L10" s="116"/>
       <c r="M10" s="55"/>
-      <c r="N10" s="91">
+      <c r="N10" s="126">
         <v>370000</v>
       </c>
-      <c r="O10" s="91"/>
-      <c r="P10" s="91"/>
+      <c r="O10" s="126"/>
+      <c r="P10" s="126"/>
       <c r="Q10" s="47"/>
       <c r="R10" s="49"/>
       <c r="S10" s="47"/>
@@ -3954,10 +3956,10 @@
       <c r="A11" s="47"/>
       <c r="B11" s="48"/>
       <c r="C11" s="47"/>
-      <c r="D11" s="107">
+      <c r="D11" s="127">
         <v>52</v>
       </c>
-      <c r="E11" s="107"/>
+      <c r="E11" s="127"/>
       <c r="F11" s="47"/>
       <c r="G11" s="47"/>
       <c r="H11" s="47"/>
@@ -3966,36 +3968,36 @@
       <c r="K11" s="47"/>
       <c r="L11" s="47"/>
       <c r="M11" s="47"/>
-      <c r="N11" s="107">
+      <c r="N11" s="127">
         <v>53</v>
       </c>
-      <c r="O11" s="107"/>
-      <c r="P11" s="107"/>
+      <c r="O11" s="127"/>
+      <c r="P11" s="127"/>
       <c r="Q11" s="47"/>
       <c r="R11" s="49"/>
       <c r="S11" s="47"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="47"/>
-      <c r="B12" s="108" t="s">
+      <c r="B12" s="118" t="s">
         <v>105</v>
       </c>
-      <c r="C12" s="109"/>
-      <c r="D12" s="109"/>
-      <c r="E12" s="109"/>
-      <c r="F12" s="109"/>
-      <c r="G12" s="109"/>
-      <c r="H12" s="109"/>
-      <c r="I12" s="109"/>
-      <c r="J12" s="109"/>
-      <c r="K12" s="109"/>
-      <c r="L12" s="109"/>
-      <c r="M12" s="109"/>
-      <c r="N12" s="109"/>
-      <c r="O12" s="109"/>
-      <c r="P12" s="109"/>
-      <c r="Q12" s="109"/>
-      <c r="R12" s="110"/>
+      <c r="C12" s="119"/>
+      <c r="D12" s="119"/>
+      <c r="E12" s="119"/>
+      <c r="F12" s="119"/>
+      <c r="G12" s="119"/>
+      <c r="H12" s="119"/>
+      <c r="I12" s="119"/>
+      <c r="J12" s="119"/>
+      <c r="K12" s="119"/>
+      <c r="L12" s="119"/>
+      <c r="M12" s="119"/>
+      <c r="N12" s="119"/>
+      <c r="O12" s="119"/>
+      <c r="P12" s="119"/>
+      <c r="Q12" s="119"/>
+      <c r="R12" s="120"/>
       <c r="S12" s="47"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.3">
@@ -4028,14 +4030,14 @@
       <c r="D14" s="47"/>
       <c r="E14" s="47"/>
       <c r="F14" s="47"/>
-      <c r="G14" s="111"/>
-      <c r="H14" s="111"/>
-      <c r="I14" s="112" t="s">
+      <c r="G14" s="128"/>
+      <c r="H14" s="128"/>
+      <c r="I14" s="125" t="s">
         <v>100</v>
       </c>
-      <c r="J14" s="112"/>
-      <c r="K14" s="113"/>
-      <c r="L14" s="113"/>
+      <c r="J14" s="125"/>
+      <c r="K14" s="129"/>
+      <c r="L14" s="129"/>
       <c r="M14" s="59"/>
       <c r="N14" s="60" t="s">
         <v>107</v>
@@ -4053,16 +4055,16 @@
       <c r="D15" s="47"/>
       <c r="E15" s="47"/>
       <c r="F15" s="47"/>
-      <c r="G15" s="103">
+      <c r="G15" s="122">
         <v>54</v>
       </c>
-      <c r="H15" s="103"/>
+      <c r="H15" s="122"/>
       <c r="I15" s="47"/>
       <c r="J15" s="47"/>
-      <c r="K15" s="103">
+      <c r="K15" s="122">
         <v>55</v>
       </c>
-      <c r="L15" s="103"/>
+      <c r="L15" s="122"/>
       <c r="M15" s="47"/>
       <c r="N15" s="47"/>
       <c r="O15" s="47"/>
@@ -4073,12 +4075,12 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="47"/>
-      <c r="B16" s="104" t="s">
+      <c r="B16" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="C16" s="105"/>
-      <c r="D16" s="91"/>
-      <c r="E16" s="91"/>
+      <c r="C16" s="115"/>
+      <c r="D16" s="126"/>
+      <c r="E16" s="126"/>
       <c r="F16" s="47"/>
       <c r="G16" s="47"/>
       <c r="H16" s="47"/>
@@ -4098,10 +4100,10 @@
       <c r="A17" s="47"/>
       <c r="B17" s="48"/>
       <c r="C17" s="61"/>
-      <c r="D17" s="103">
+      <c r="D17" s="122">
         <v>56</v>
       </c>
-      <c r="E17" s="103"/>
+      <c r="E17" s="122"/>
       <c r="F17" s="47"/>
       <c r="G17" s="47"/>
       <c r="H17" s="47"/>
@@ -4119,25 +4121,25 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="47"/>
-      <c r="B18" s="104" t="s">
+      <c r="B18" s="123" t="s">
         <v>103</v>
       </c>
-      <c r="C18" s="105"/>
-      <c r="D18" s="106"/>
-      <c r="E18" s="106"/>
+      <c r="C18" s="115"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="124"/>
       <c r="F18" s="47"/>
       <c r="G18" s="47"/>
       <c r="H18" s="47"/>
       <c r="I18" s="47"/>
       <c r="J18" s="47"/>
-      <c r="K18" s="105" t="s">
+      <c r="K18" s="115" t="s">
         <v>102</v>
       </c>
-      <c r="L18" s="105"/>
-      <c r="M18" s="105"/>
-      <c r="N18" s="91"/>
-      <c r="O18" s="91"/>
-      <c r="P18" s="91"/>
+      <c r="L18" s="115"/>
+      <c r="M18" s="115"/>
+      <c r="N18" s="126"/>
+      <c r="O18" s="126"/>
+      <c r="P18" s="126"/>
       <c r="Q18" s="47"/>
       <c r="R18" s="49"/>
       <c r="S18" s="47"/>
@@ -4171,71 +4173,71 @@
       <c r="A20" s="47">
         <v>36</v>
       </c>
-      <c r="B20" s="92" t="s">
+      <c r="B20" s="133" t="s">
         <v>108</v>
       </c>
-      <c r="C20" s="93"/>
-      <c r="D20" s="94"/>
-      <c r="E20" s="95"/>
-      <c r="F20" s="95"/>
-      <c r="G20" s="95"/>
-      <c r="H20" s="95"/>
-      <c r="I20" s="95"/>
-      <c r="J20" s="95"/>
-      <c r="K20" s="95"/>
-      <c r="L20" s="95"/>
-      <c r="M20" s="95"/>
-      <c r="N20" s="95"/>
-      <c r="O20" s="95"/>
-      <c r="P20" s="95"/>
-      <c r="Q20" s="95"/>
-      <c r="R20" s="96"/>
+      <c r="C20" s="134"/>
+      <c r="D20" s="135"/>
+      <c r="E20" s="136"/>
+      <c r="F20" s="136"/>
+      <c r="G20" s="136"/>
+      <c r="H20" s="136"/>
+      <c r="I20" s="136"/>
+      <c r="J20" s="136"/>
+      <c r="K20" s="136"/>
+      <c r="L20" s="136"/>
+      <c r="M20" s="136"/>
+      <c r="N20" s="136"/>
+      <c r="O20" s="136"/>
+      <c r="P20" s="136"/>
+      <c r="Q20" s="136"/>
+      <c r="R20" s="137"/>
       <c r="S20" s="47"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="47">
         <v>90</v>
       </c>
-      <c r="B21" s="80"/>
-      <c r="C21" s="81"/>
-      <c r="D21" s="81"/>
-      <c r="E21" s="81"/>
-      <c r="F21" s="81"/>
-      <c r="G21" s="81"/>
-      <c r="H21" s="81"/>
-      <c r="I21" s="81"/>
-      <c r="J21" s="81"/>
-      <c r="K21" s="81"/>
-      <c r="L21" s="81"/>
-      <c r="M21" s="81"/>
-      <c r="N21" s="81"/>
-      <c r="O21" s="81"/>
-      <c r="P21" s="81"/>
-      <c r="Q21" s="81"/>
-      <c r="R21" s="82"/>
+      <c r="B21" s="130"/>
+      <c r="C21" s="131"/>
+      <c r="D21" s="131"/>
+      <c r="E21" s="131"/>
+      <c r="F21" s="131"/>
+      <c r="G21" s="131"/>
+      <c r="H21" s="131"/>
+      <c r="I21" s="131"/>
+      <c r="J21" s="131"/>
+      <c r="K21" s="131"/>
+      <c r="L21" s="131"/>
+      <c r="M21" s="131"/>
+      <c r="N21" s="131"/>
+      <c r="O21" s="131"/>
+      <c r="P21" s="131"/>
+      <c r="Q21" s="131"/>
+      <c r="R21" s="132"/>
       <c r="S21" s="47"/>
     </row>
     <row r="22" spans="1:19" ht="15" x14ac:dyDescent="0.3">
       <c r="A22" s="47">
         <v>101</v>
       </c>
-      <c r="B22" s="97"/>
-      <c r="C22" s="98"/>
-      <c r="D22" s="98"/>
-      <c r="E22" s="98"/>
-      <c r="F22" s="98"/>
-      <c r="G22" s="98"/>
-      <c r="H22" s="98"/>
-      <c r="I22" s="98"/>
-      <c r="J22" s="98"/>
-      <c r="K22" s="98"/>
-      <c r="L22" s="98"/>
-      <c r="M22" s="98"/>
-      <c r="N22" s="98"/>
-      <c r="O22" s="98"/>
-      <c r="P22" s="98"/>
-      <c r="Q22" s="98"/>
-      <c r="R22" s="99"/>
+      <c r="B22" s="138"/>
+      <c r="C22" s="139"/>
+      <c r="D22" s="139"/>
+      <c r="E22" s="139"/>
+      <c r="F22" s="139"/>
+      <c r="G22" s="139"/>
+      <c r="H22" s="139"/>
+      <c r="I22" s="139"/>
+      <c r="J22" s="139"/>
+      <c r="K22" s="139"/>
+      <c r="L22" s="139"/>
+      <c r="M22" s="139"/>
+      <c r="N22" s="139"/>
+      <c r="O22" s="139"/>
+      <c r="P22" s="139"/>
+      <c r="Q22" s="139"/>
+      <c r="R22" s="140"/>
       <c r="S22" s="47"/>
     </row>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -4282,493 +4284,493 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" s="47"/>
-      <c r="B25" s="100"/>
-      <c r="C25" s="101"/>
-      <c r="D25" s="101"/>
-      <c r="E25" s="101"/>
-      <c r="F25" s="101"/>
-      <c r="G25" s="101"/>
-      <c r="H25" s="101"/>
-      <c r="I25" s="101"/>
-      <c r="J25" s="101"/>
-      <c r="K25" s="101"/>
-      <c r="L25" s="101"/>
-      <c r="M25" s="101"/>
-      <c r="N25" s="101"/>
-      <c r="O25" s="101"/>
-      <c r="P25" s="101"/>
-      <c r="Q25" s="101"/>
-      <c r="R25" s="102"/>
+      <c r="B25" s="141"/>
+      <c r="C25" s="142"/>
+      <c r="D25" s="142"/>
+      <c r="E25" s="142"/>
+      <c r="F25" s="142"/>
+      <c r="G25" s="142"/>
+      <c r="H25" s="142"/>
+      <c r="I25" s="142"/>
+      <c r="J25" s="142"/>
+      <c r="K25" s="142"/>
+      <c r="L25" s="142"/>
+      <c r="M25" s="142"/>
+      <c r="N25" s="142"/>
+      <c r="O25" s="142"/>
+      <c r="P25" s="142"/>
+      <c r="Q25" s="142"/>
+      <c r="R25" s="143"/>
       <c r="S25" s="47"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" s="47"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="81"/>
-      <c r="D26" s="81"/>
-      <c r="E26" s="81"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="81"/>
-      <c r="H26" s="81"/>
-      <c r="I26" s="81"/>
-      <c r="J26" s="81"/>
-      <c r="K26" s="81"/>
-      <c r="L26" s="81"/>
-      <c r="M26" s="81"/>
-      <c r="N26" s="81"/>
-      <c r="O26" s="81"/>
-      <c r="P26" s="81"/>
-      <c r="Q26" s="81"/>
-      <c r="R26" s="82"/>
+      <c r="B26" s="130"/>
+      <c r="C26" s="131"/>
+      <c r="D26" s="131"/>
+      <c r="E26" s="131"/>
+      <c r="F26" s="131"/>
+      <c r="G26" s="131"/>
+      <c r="H26" s="131"/>
+      <c r="I26" s="131"/>
+      <c r="J26" s="131"/>
+      <c r="K26" s="131"/>
+      <c r="L26" s="131"/>
+      <c r="M26" s="131"/>
+      <c r="N26" s="131"/>
+      <c r="O26" s="131"/>
+      <c r="P26" s="131"/>
+      <c r="Q26" s="131"/>
+      <c r="R26" s="132"/>
       <c r="S26" s="47"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" s="47"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="81"/>
-      <c r="D27" s="81"/>
-      <c r="E27" s="81"/>
-      <c r="F27" s="81"/>
-      <c r="G27" s="81"/>
-      <c r="H27" s="81"/>
-      <c r="I27" s="81"/>
-      <c r="J27" s="81"/>
-      <c r="K27" s="81"/>
-      <c r="L27" s="81"/>
-      <c r="M27" s="81"/>
-      <c r="N27" s="81"/>
-      <c r="O27" s="81"/>
-      <c r="P27" s="81"/>
-      <c r="Q27" s="81"/>
-      <c r="R27" s="82"/>
+      <c r="B27" s="130"/>
+      <c r="C27" s="131"/>
+      <c r="D27" s="131"/>
+      <c r="E27" s="131"/>
+      <c r="F27" s="131"/>
+      <c r="G27" s="131"/>
+      <c r="H27" s="131"/>
+      <c r="I27" s="131"/>
+      <c r="J27" s="131"/>
+      <c r="K27" s="131"/>
+      <c r="L27" s="131"/>
+      <c r="M27" s="131"/>
+      <c r="N27" s="131"/>
+      <c r="O27" s="131"/>
+      <c r="P27" s="131"/>
+      <c r="Q27" s="131"/>
+      <c r="R27" s="132"/>
       <c r="S27" s="47"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" s="47"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="81"/>
-      <c r="D28" s="81"/>
-      <c r="E28" s="81"/>
-      <c r="F28" s="81"/>
-      <c r="G28" s="81"/>
-      <c r="H28" s="81"/>
-      <c r="I28" s="81"/>
-      <c r="J28" s="81"/>
-      <c r="K28" s="81"/>
-      <c r="L28" s="81"/>
-      <c r="M28" s="81"/>
-      <c r="N28" s="81"/>
-      <c r="O28" s="81"/>
-      <c r="P28" s="81"/>
-      <c r="Q28" s="81"/>
-      <c r="R28" s="82"/>
+      <c r="B28" s="130"/>
+      <c r="C28" s="131"/>
+      <c r="D28" s="131"/>
+      <c r="E28" s="131"/>
+      <c r="F28" s="131"/>
+      <c r="G28" s="131"/>
+      <c r="H28" s="131"/>
+      <c r="I28" s="131"/>
+      <c r="J28" s="131"/>
+      <c r="K28" s="131"/>
+      <c r="L28" s="131"/>
+      <c r="M28" s="131"/>
+      <c r="N28" s="131"/>
+      <c r="O28" s="131"/>
+      <c r="P28" s="131"/>
+      <c r="Q28" s="131"/>
+      <c r="R28" s="132"/>
       <c r="S28" s="47"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" s="47"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="81"/>
-      <c r="D29" s="81"/>
-      <c r="E29" s="81"/>
-      <c r="F29" s="81"/>
-      <c r="G29" s="81"/>
-      <c r="H29" s="81"/>
-      <c r="I29" s="81"/>
-      <c r="J29" s="81"/>
-      <c r="K29" s="81"/>
-      <c r="L29" s="81"/>
-      <c r="M29" s="81"/>
-      <c r="N29" s="81"/>
-      <c r="O29" s="81"/>
-      <c r="P29" s="81"/>
-      <c r="Q29" s="81"/>
-      <c r="R29" s="82"/>
+      <c r="B29" s="130"/>
+      <c r="C29" s="131"/>
+      <c r="D29" s="131"/>
+      <c r="E29" s="131"/>
+      <c r="F29" s="131"/>
+      <c r="G29" s="131"/>
+      <c r="H29" s="131"/>
+      <c r="I29" s="131"/>
+      <c r="J29" s="131"/>
+      <c r="K29" s="131"/>
+      <c r="L29" s="131"/>
+      <c r="M29" s="131"/>
+      <c r="N29" s="131"/>
+      <c r="O29" s="131"/>
+      <c r="P29" s="131"/>
+      <c r="Q29" s="131"/>
+      <c r="R29" s="132"/>
       <c r="S29" s="47"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="47"/>
-      <c r="B30" s="88"/>
-      <c r="C30" s="89"/>
-      <c r="D30" s="89"/>
-      <c r="E30" s="89"/>
-      <c r="F30" s="89"/>
-      <c r="G30" s="89"/>
-      <c r="H30" s="89"/>
-      <c r="I30" s="89"/>
-      <c r="J30" s="89"/>
-      <c r="K30" s="89"/>
-      <c r="L30" s="89"/>
-      <c r="M30" s="89"/>
-      <c r="N30" s="89"/>
-      <c r="O30" s="89"/>
-      <c r="P30" s="89"/>
-      <c r="Q30" s="89"/>
-      <c r="R30" s="90"/>
+      <c r="B30" s="144"/>
+      <c r="C30" s="145"/>
+      <c r="D30" s="145"/>
+      <c r="E30" s="145"/>
+      <c r="F30" s="145"/>
+      <c r="G30" s="145"/>
+      <c r="H30" s="145"/>
+      <c r="I30" s="145"/>
+      <c r="J30" s="145"/>
+      <c r="K30" s="145"/>
+      <c r="L30" s="145"/>
+      <c r="M30" s="145"/>
+      <c r="N30" s="145"/>
+      <c r="O30" s="145"/>
+      <c r="P30" s="145"/>
+      <c r="Q30" s="145"/>
+      <c r="R30" s="146"/>
       <c r="S30" s="47"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" s="47"/>
-      <c r="B31" s="80"/>
-      <c r="C31" s="81"/>
-      <c r="D31" s="81"/>
-      <c r="E31" s="81"/>
-      <c r="F31" s="81"/>
-      <c r="G31" s="81"/>
-      <c r="H31" s="81"/>
-      <c r="I31" s="81"/>
-      <c r="J31" s="81"/>
-      <c r="K31" s="81"/>
-      <c r="L31" s="81"/>
-      <c r="M31" s="81"/>
-      <c r="N31" s="81"/>
-      <c r="O31" s="81"/>
-      <c r="P31" s="81"/>
-      <c r="Q31" s="81"/>
-      <c r="R31" s="82"/>
+      <c r="B31" s="130"/>
+      <c r="C31" s="131"/>
+      <c r="D31" s="131"/>
+      <c r="E31" s="131"/>
+      <c r="F31" s="131"/>
+      <c r="G31" s="131"/>
+      <c r="H31" s="131"/>
+      <c r="I31" s="131"/>
+      <c r="J31" s="131"/>
+      <c r="K31" s="131"/>
+      <c r="L31" s="131"/>
+      <c r="M31" s="131"/>
+      <c r="N31" s="131"/>
+      <c r="O31" s="131"/>
+      <c r="P31" s="131"/>
+      <c r="Q31" s="131"/>
+      <c r="R31" s="132"/>
       <c r="S31" s="47"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A32" s="47"/>
-      <c r="B32" s="80"/>
-      <c r="C32" s="81"/>
-      <c r="D32" s="81"/>
-      <c r="E32" s="81"/>
-      <c r="F32" s="81"/>
-      <c r="G32" s="81"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="81"/>
-      <c r="J32" s="81"/>
-      <c r="K32" s="81"/>
-      <c r="L32" s="81"/>
-      <c r="M32" s="81"/>
-      <c r="N32" s="81"/>
-      <c r="O32" s="81"/>
-      <c r="P32" s="81"/>
-      <c r="Q32" s="81"/>
-      <c r="R32" s="82"/>
+      <c r="B32" s="130"/>
+      <c r="C32" s="131"/>
+      <c r="D32" s="131"/>
+      <c r="E32" s="131"/>
+      <c r="F32" s="131"/>
+      <c r="G32" s="131"/>
+      <c r="H32" s="131"/>
+      <c r="I32" s="131"/>
+      <c r="J32" s="131"/>
+      <c r="K32" s="131"/>
+      <c r="L32" s="131"/>
+      <c r="M32" s="131"/>
+      <c r="N32" s="131"/>
+      <c r="O32" s="131"/>
+      <c r="P32" s="131"/>
+      <c r="Q32" s="131"/>
+      <c r="R32" s="132"/>
       <c r="S32" s="47"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" s="47"/>
-      <c r="B33" s="80"/>
-      <c r="C33" s="81"/>
-      <c r="D33" s="81"/>
-      <c r="E33" s="81"/>
-      <c r="F33" s="81"/>
-      <c r="G33" s="81"/>
-      <c r="H33" s="81"/>
-      <c r="I33" s="81"/>
-      <c r="J33" s="81"/>
-      <c r="K33" s="81"/>
-      <c r="L33" s="81"/>
-      <c r="M33" s="81"/>
-      <c r="N33" s="81"/>
-      <c r="O33" s="81"/>
-      <c r="P33" s="81"/>
-      <c r="Q33" s="81"/>
-      <c r="R33" s="82"/>
+      <c r="B33" s="130"/>
+      <c r="C33" s="131"/>
+      <c r="D33" s="131"/>
+      <c r="E33" s="131"/>
+      <c r="F33" s="131"/>
+      <c r="G33" s="131"/>
+      <c r="H33" s="131"/>
+      <c r="I33" s="131"/>
+      <c r="J33" s="131"/>
+      <c r="K33" s="131"/>
+      <c r="L33" s="131"/>
+      <c r="M33" s="131"/>
+      <c r="N33" s="131"/>
+      <c r="O33" s="131"/>
+      <c r="P33" s="131"/>
+      <c r="Q33" s="131"/>
+      <c r="R33" s="132"/>
       <c r="S33" s="47"/>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A34" s="47"/>
-      <c r="B34" s="85"/>
-      <c r="C34" s="86"/>
-      <c r="D34" s="86"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="86"/>
-      <c r="G34" s="86"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="86"/>
-      <c r="J34" s="86"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="86"/>
-      <c r="M34" s="86"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="86"/>
-      <c r="P34" s="86"/>
-      <c r="Q34" s="86"/>
-      <c r="R34" s="87"/>
+      <c r="B34" s="147"/>
+      <c r="C34" s="148"/>
+      <c r="D34" s="148"/>
+      <c r="E34" s="148"/>
+      <c r="F34" s="148"/>
+      <c r="G34" s="148"/>
+      <c r="H34" s="148"/>
+      <c r="I34" s="148"/>
+      <c r="J34" s="148"/>
+      <c r="K34" s="148"/>
+      <c r="L34" s="148"/>
+      <c r="M34" s="148"/>
+      <c r="N34" s="148"/>
+      <c r="O34" s="148"/>
+      <c r="P34" s="148"/>
+      <c r="Q34" s="148"/>
+      <c r="R34" s="149"/>
       <c r="S34" s="47"/>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" s="47"/>
-      <c r="B35" s="88"/>
-      <c r="C35" s="89"/>
-      <c r="D35" s="89"/>
-      <c r="E35" s="89"/>
-      <c r="F35" s="89"/>
-      <c r="G35" s="89"/>
-      <c r="H35" s="89"/>
-      <c r="I35" s="89"/>
-      <c r="J35" s="89"/>
-      <c r="K35" s="89"/>
-      <c r="L35" s="89"/>
-      <c r="M35" s="89"/>
-      <c r="N35" s="89"/>
-      <c r="O35" s="89"/>
-      <c r="P35" s="89"/>
-      <c r="Q35" s="89"/>
-      <c r="R35" s="90"/>
+      <c r="B35" s="144"/>
+      <c r="C35" s="145"/>
+      <c r="D35" s="145"/>
+      <c r="E35" s="145"/>
+      <c r="F35" s="145"/>
+      <c r="G35" s="145"/>
+      <c r="H35" s="145"/>
+      <c r="I35" s="145"/>
+      <c r="J35" s="145"/>
+      <c r="K35" s="145"/>
+      <c r="L35" s="145"/>
+      <c r="M35" s="145"/>
+      <c r="N35" s="145"/>
+      <c r="O35" s="145"/>
+      <c r="P35" s="145"/>
+      <c r="Q35" s="145"/>
+      <c r="R35" s="146"/>
       <c r="S35" s="47"/>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" s="47"/>
-      <c r="B36" s="80"/>
-      <c r="C36" s="81"/>
-      <c r="D36" s="81"/>
-      <c r="E36" s="81"/>
-      <c r="F36" s="81"/>
-      <c r="G36" s="81"/>
-      <c r="H36" s="81"/>
-      <c r="I36" s="81"/>
-      <c r="J36" s="81"/>
-      <c r="K36" s="81"/>
-      <c r="L36" s="81"/>
-      <c r="M36" s="81"/>
-      <c r="N36" s="81"/>
-      <c r="O36" s="81"/>
-      <c r="P36" s="81"/>
-      <c r="Q36" s="81"/>
-      <c r="R36" s="82"/>
+      <c r="B36" s="130"/>
+      <c r="C36" s="131"/>
+      <c r="D36" s="131"/>
+      <c r="E36" s="131"/>
+      <c r="F36" s="131"/>
+      <c r="G36" s="131"/>
+      <c r="H36" s="131"/>
+      <c r="I36" s="131"/>
+      <c r="J36" s="131"/>
+      <c r="K36" s="131"/>
+      <c r="L36" s="131"/>
+      <c r="M36" s="131"/>
+      <c r="N36" s="131"/>
+      <c r="O36" s="131"/>
+      <c r="P36" s="131"/>
+      <c r="Q36" s="131"/>
+      <c r="R36" s="132"/>
       <c r="S36" s="47"/>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" s="47"/>
-      <c r="B37" s="80"/>
-      <c r="C37" s="81"/>
-      <c r="D37" s="81"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="81"/>
-      <c r="G37" s="81"/>
-      <c r="H37" s="81"/>
-      <c r="I37" s="81"/>
-      <c r="J37" s="81"/>
-      <c r="K37" s="81"/>
-      <c r="L37" s="81"/>
-      <c r="M37" s="81"/>
-      <c r="N37" s="81"/>
-      <c r="O37" s="81"/>
-      <c r="P37" s="81"/>
-      <c r="Q37" s="81"/>
-      <c r="R37" s="82"/>
+      <c r="B37" s="130"/>
+      <c r="C37" s="131"/>
+      <c r="D37" s="131"/>
+      <c r="E37" s="131"/>
+      <c r="F37" s="131"/>
+      <c r="G37" s="131"/>
+      <c r="H37" s="131"/>
+      <c r="I37" s="131"/>
+      <c r="J37" s="131"/>
+      <c r="K37" s="131"/>
+      <c r="L37" s="131"/>
+      <c r="M37" s="131"/>
+      <c r="N37" s="131"/>
+      <c r="O37" s="131"/>
+      <c r="P37" s="131"/>
+      <c r="Q37" s="131"/>
+      <c r="R37" s="132"/>
       <c r="S37" s="47"/>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" s="47"/>
-      <c r="B38" s="80"/>
-      <c r="C38" s="81"/>
-      <c r="D38" s="81"/>
-      <c r="E38" s="81"/>
-      <c r="F38" s="81"/>
-      <c r="G38" s="81"/>
-      <c r="H38" s="81"/>
-      <c r="I38" s="81"/>
-      <c r="J38" s="81"/>
-      <c r="K38" s="81"/>
-      <c r="L38" s="81"/>
-      <c r="M38" s="81"/>
-      <c r="N38" s="81"/>
-      <c r="O38" s="81"/>
-      <c r="P38" s="81"/>
-      <c r="Q38" s="81"/>
-      <c r="R38" s="82"/>
+      <c r="B38" s="130"/>
+      <c r="C38" s="131"/>
+      <c r="D38" s="131"/>
+      <c r="E38" s="131"/>
+      <c r="F38" s="131"/>
+      <c r="G38" s="131"/>
+      <c r="H38" s="131"/>
+      <c r="I38" s="131"/>
+      <c r="J38" s="131"/>
+      <c r="K38" s="131"/>
+      <c r="L38" s="131"/>
+      <c r="M38" s="131"/>
+      <c r="N38" s="131"/>
+      <c r="O38" s="131"/>
+      <c r="P38" s="131"/>
+      <c r="Q38" s="131"/>
+      <c r="R38" s="132"/>
       <c r="S38" s="47"/>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" s="47"/>
-      <c r="B39" s="80"/>
-      <c r="C39" s="81"/>
-      <c r="D39" s="81"/>
-      <c r="E39" s="81"/>
-      <c r="F39" s="81"/>
-      <c r="G39" s="81"/>
-      <c r="H39" s="81"/>
-      <c r="I39" s="81"/>
-      <c r="J39" s="81"/>
-      <c r="K39" s="81"/>
-      <c r="L39" s="81"/>
-      <c r="M39" s="81"/>
-      <c r="N39" s="81"/>
-      <c r="O39" s="81"/>
-      <c r="P39" s="81"/>
-      <c r="Q39" s="81"/>
-      <c r="R39" s="82"/>
+      <c r="B39" s="130"/>
+      <c r="C39" s="131"/>
+      <c r="D39" s="131"/>
+      <c r="E39" s="131"/>
+      <c r="F39" s="131"/>
+      <c r="G39" s="131"/>
+      <c r="H39" s="131"/>
+      <c r="I39" s="131"/>
+      <c r="J39" s="131"/>
+      <c r="K39" s="131"/>
+      <c r="L39" s="131"/>
+      <c r="M39" s="131"/>
+      <c r="N39" s="131"/>
+      <c r="O39" s="131"/>
+      <c r="P39" s="131"/>
+      <c r="Q39" s="131"/>
+      <c r="R39" s="132"/>
       <c r="S39" s="47"/>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" s="47"/>
-      <c r="B40" s="80"/>
-      <c r="C40" s="81"/>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="81"/>
-      <c r="H40" s="81"/>
-      <c r="I40" s="81"/>
-      <c r="J40" s="81"/>
-      <c r="K40" s="81"/>
-      <c r="L40" s="81"/>
-      <c r="M40" s="81"/>
-      <c r="N40" s="81"/>
-      <c r="O40" s="81"/>
-      <c r="P40" s="81"/>
-      <c r="Q40" s="81"/>
-      <c r="R40" s="82"/>
+      <c r="B40" s="130"/>
+      <c r="C40" s="131"/>
+      <c r="D40" s="131"/>
+      <c r="E40" s="131"/>
+      <c r="F40" s="131"/>
+      <c r="G40" s="131"/>
+      <c r="H40" s="131"/>
+      <c r="I40" s="131"/>
+      <c r="J40" s="131"/>
+      <c r="K40" s="131"/>
+      <c r="L40" s="131"/>
+      <c r="M40" s="131"/>
+      <c r="N40" s="131"/>
+      <c r="O40" s="131"/>
+      <c r="P40" s="131"/>
+      <c r="Q40" s="131"/>
+      <c r="R40" s="132"/>
       <c r="S40" s="47"/>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" s="47"/>
-      <c r="B41" s="80"/>
-      <c r="C41" s="81"/>
-      <c r="D41" s="81"/>
-      <c r="E41" s="81"/>
-      <c r="F41" s="81"/>
-      <c r="G41" s="81"/>
-      <c r="H41" s="81"/>
-      <c r="I41" s="81"/>
-      <c r="J41" s="81"/>
-      <c r="K41" s="81"/>
-      <c r="L41" s="81"/>
-      <c r="M41" s="81"/>
-      <c r="N41" s="81"/>
-      <c r="O41" s="81"/>
-      <c r="P41" s="81"/>
-      <c r="Q41" s="81"/>
-      <c r="R41" s="82"/>
+      <c r="B41" s="130"/>
+      <c r="C41" s="131"/>
+      <c r="D41" s="131"/>
+      <c r="E41" s="131"/>
+      <c r="F41" s="131"/>
+      <c r="G41" s="131"/>
+      <c r="H41" s="131"/>
+      <c r="I41" s="131"/>
+      <c r="J41" s="131"/>
+      <c r="K41" s="131"/>
+      <c r="L41" s="131"/>
+      <c r="M41" s="131"/>
+      <c r="N41" s="131"/>
+      <c r="O41" s="131"/>
+      <c r="P41" s="131"/>
+      <c r="Q41" s="131"/>
+      <c r="R41" s="132"/>
       <c r="S41" s="47"/>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" s="47"/>
-      <c r="B42" s="80"/>
-      <c r="C42" s="81"/>
-      <c r="D42" s="81"/>
-      <c r="E42" s="81"/>
-      <c r="F42" s="81"/>
-      <c r="G42" s="81"/>
-      <c r="H42" s="81"/>
-      <c r="I42" s="81"/>
-      <c r="J42" s="81"/>
-      <c r="K42" s="81"/>
-      <c r="L42" s="81"/>
-      <c r="M42" s="81"/>
-      <c r="N42" s="81"/>
-      <c r="O42" s="81"/>
-      <c r="P42" s="81"/>
-      <c r="Q42" s="81"/>
-      <c r="R42" s="82"/>
+      <c r="B42" s="130"/>
+      <c r="C42" s="131"/>
+      <c r="D42" s="131"/>
+      <c r="E42" s="131"/>
+      <c r="F42" s="131"/>
+      <c r="G42" s="131"/>
+      <c r="H42" s="131"/>
+      <c r="I42" s="131"/>
+      <c r="J42" s="131"/>
+      <c r="K42" s="131"/>
+      <c r="L42" s="131"/>
+      <c r="M42" s="131"/>
+      <c r="N42" s="131"/>
+      <c r="O42" s="131"/>
+      <c r="P42" s="131"/>
+      <c r="Q42" s="131"/>
+      <c r="R42" s="132"/>
       <c r="S42" s="47"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" s="47"/>
-      <c r="B43" s="80"/>
-      <c r="C43" s="81"/>
-      <c r="D43" s="81"/>
-      <c r="E43" s="81"/>
-      <c r="F43" s="81"/>
-      <c r="G43" s="81"/>
-      <c r="H43" s="81"/>
-      <c r="I43" s="81"/>
-      <c r="J43" s="81"/>
-      <c r="K43" s="81"/>
-      <c r="L43" s="81"/>
-      <c r="M43" s="81"/>
-      <c r="N43" s="81"/>
-      <c r="O43" s="81"/>
-      <c r="P43" s="81"/>
-      <c r="Q43" s="81"/>
-      <c r="R43" s="82"/>
+      <c r="B43" s="130"/>
+      <c r="C43" s="131"/>
+      <c r="D43" s="131"/>
+      <c r="E43" s="131"/>
+      <c r="F43" s="131"/>
+      <c r="G43" s="131"/>
+      <c r="H43" s="131"/>
+      <c r="I43" s="131"/>
+      <c r="J43" s="131"/>
+      <c r="K43" s="131"/>
+      <c r="L43" s="131"/>
+      <c r="M43" s="131"/>
+      <c r="N43" s="131"/>
+      <c r="O43" s="131"/>
+      <c r="P43" s="131"/>
+      <c r="Q43" s="131"/>
+      <c r="R43" s="132"/>
       <c r="S43" s="47"/>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" s="47"/>
-      <c r="B44" s="80"/>
-      <c r="C44" s="81"/>
-      <c r="D44" s="81"/>
-      <c r="E44" s="81"/>
-      <c r="F44" s="81"/>
-      <c r="G44" s="81"/>
-      <c r="H44" s="81"/>
-      <c r="I44" s="81"/>
-      <c r="J44" s="81"/>
-      <c r="K44" s="81"/>
-      <c r="L44" s="81"/>
-      <c r="M44" s="81"/>
-      <c r="N44" s="81"/>
-      <c r="O44" s="81"/>
-      <c r="P44" s="81"/>
-      <c r="Q44" s="81"/>
-      <c r="R44" s="82"/>
+      <c r="B44" s="130"/>
+      <c r="C44" s="131"/>
+      <c r="D44" s="131"/>
+      <c r="E44" s="131"/>
+      <c r="F44" s="131"/>
+      <c r="G44" s="131"/>
+      <c r="H44" s="131"/>
+      <c r="I44" s="131"/>
+      <c r="J44" s="131"/>
+      <c r="K44" s="131"/>
+      <c r="L44" s="131"/>
+      <c r="M44" s="131"/>
+      <c r="N44" s="131"/>
+      <c r="O44" s="131"/>
+      <c r="P44" s="131"/>
+      <c r="Q44" s="131"/>
+      <c r="R44" s="132"/>
       <c r="S44" s="47"/>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" s="47"/>
-      <c r="B45" s="80"/>
-      <c r="C45" s="81"/>
-      <c r="D45" s="81"/>
-      <c r="E45" s="81"/>
-      <c r="F45" s="81"/>
-      <c r="G45" s="81"/>
-      <c r="H45" s="81"/>
-      <c r="I45" s="81"/>
-      <c r="J45" s="81"/>
-      <c r="K45" s="81"/>
-      <c r="L45" s="81"/>
-      <c r="M45" s="81"/>
-      <c r="N45" s="81"/>
-      <c r="O45" s="81"/>
-      <c r="P45" s="81"/>
-      <c r="Q45" s="81"/>
-      <c r="R45" s="82"/>
+      <c r="B45" s="130"/>
+      <c r="C45" s="131"/>
+      <c r="D45" s="131"/>
+      <c r="E45" s="131"/>
+      <c r="F45" s="131"/>
+      <c r="G45" s="131"/>
+      <c r="H45" s="131"/>
+      <c r="I45" s="131"/>
+      <c r="J45" s="131"/>
+      <c r="K45" s="131"/>
+      <c r="L45" s="131"/>
+      <c r="M45" s="131"/>
+      <c r="N45" s="131"/>
+      <c r="O45" s="131"/>
+      <c r="P45" s="131"/>
+      <c r="Q45" s="131"/>
+      <c r="R45" s="132"/>
       <c r="S45" s="47"/>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" s="47"/>
-      <c r="B46" s="80"/>
-      <c r="C46" s="81"/>
-      <c r="D46" s="81"/>
-      <c r="E46" s="81"/>
-      <c r="F46" s="81"/>
-      <c r="G46" s="81"/>
-      <c r="H46" s="81"/>
-      <c r="I46" s="81"/>
-      <c r="J46" s="81"/>
-      <c r="K46" s="81"/>
-      <c r="L46" s="81"/>
-      <c r="M46" s="81"/>
-      <c r="N46" s="81"/>
-      <c r="O46" s="81"/>
-      <c r="P46" s="81"/>
-      <c r="Q46" s="81"/>
-      <c r="R46" s="82"/>
+      <c r="B46" s="130"/>
+      <c r="C46" s="131"/>
+      <c r="D46" s="131"/>
+      <c r="E46" s="131"/>
+      <c r="F46" s="131"/>
+      <c r="G46" s="131"/>
+      <c r="H46" s="131"/>
+      <c r="I46" s="131"/>
+      <c r="J46" s="131"/>
+      <c r="K46" s="131"/>
+      <c r="L46" s="131"/>
+      <c r="M46" s="131"/>
+      <c r="N46" s="131"/>
+      <c r="O46" s="131"/>
+      <c r="P46" s="131"/>
+      <c r="Q46" s="131"/>
+      <c r="R46" s="132"/>
       <c r="S46" s="47"/>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A47" s="47"/>
-      <c r="B47" s="80"/>
-      <c r="C47" s="81"/>
-      <c r="D47" s="81"/>
-      <c r="E47" s="81"/>
-      <c r="F47" s="81"/>
-      <c r="G47" s="81"/>
-      <c r="H47" s="81"/>
-      <c r="I47" s="81"/>
-      <c r="J47" s="81"/>
-      <c r="K47" s="81"/>
-      <c r="L47" s="81"/>
-      <c r="M47" s="81"/>
-      <c r="N47" s="81"/>
-      <c r="O47" s="81"/>
-      <c r="P47" s="81"/>
-      <c r="Q47" s="81"/>
-      <c r="R47" s="82"/>
+      <c r="B47" s="130"/>
+      <c r="C47" s="131"/>
+      <c r="D47" s="131"/>
+      <c r="E47" s="131"/>
+      <c r="F47" s="131"/>
+      <c r="G47" s="131"/>
+      <c r="H47" s="131"/>
+      <c r="I47" s="131"/>
+      <c r="J47" s="131"/>
+      <c r="K47" s="131"/>
+      <c r="L47" s="131"/>
+      <c r="M47" s="131"/>
+      <c r="N47" s="131"/>
+      <c r="O47" s="131"/>
+      <c r="P47" s="131"/>
+      <c r="Q47" s="131"/>
+      <c r="R47" s="132"/>
       <c r="S47" s="47"/>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" s="47"/>
-      <c r="B48" s="83" t="s">
+      <c r="B48" s="150" t="s">
         <v>109</v>
       </c>
-      <c r="C48" s="84"/>
+      <c r="C48" s="151"/>
       <c r="D48" s="66"/>
       <c r="E48" s="66"/>
       <c r="F48" s="66"/>
@@ -4892,34 +4894,23 @@
     </row>
   </sheetData>
   <mergeCells count="60">
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="B4:R4"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="B12:R12"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="B44:R44"/>
+    <mergeCell ref="B45:R45"/>
+    <mergeCell ref="B46:R46"/>
+    <mergeCell ref="B47:R47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B43:R43"/>
+    <mergeCell ref="B32:R32"/>
+    <mergeCell ref="B33:R33"/>
+    <mergeCell ref="B34:R34"/>
+    <mergeCell ref="B35:R35"/>
+    <mergeCell ref="B36:R36"/>
+    <mergeCell ref="B37:R37"/>
+    <mergeCell ref="B38:R38"/>
+    <mergeCell ref="B39:R39"/>
+    <mergeCell ref="B40:R40"/>
+    <mergeCell ref="B41:R41"/>
+    <mergeCell ref="B42:R42"/>
     <mergeCell ref="B31:R31"/>
     <mergeCell ref="N18:P18"/>
     <mergeCell ref="B20:C20"/>
@@ -4935,23 +4926,34 @@
     <mergeCell ref="B28:R28"/>
     <mergeCell ref="B29:R29"/>
     <mergeCell ref="B30:R30"/>
-    <mergeCell ref="B43:R43"/>
-    <mergeCell ref="B32:R32"/>
-    <mergeCell ref="B33:R33"/>
-    <mergeCell ref="B34:R34"/>
-    <mergeCell ref="B35:R35"/>
-    <mergeCell ref="B36:R36"/>
-    <mergeCell ref="B37:R37"/>
-    <mergeCell ref="B38:R38"/>
-    <mergeCell ref="B39:R39"/>
-    <mergeCell ref="B40:R40"/>
-    <mergeCell ref="B41:R41"/>
-    <mergeCell ref="B42:R42"/>
-    <mergeCell ref="B44:R44"/>
-    <mergeCell ref="B45:R45"/>
-    <mergeCell ref="B46:R46"/>
-    <mergeCell ref="B47:R47"/>
-    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="B12:R12"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="B4:R4"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="K7:L7"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.25" bottom="0" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix(reporte): merge cells B23:R35 for remarks on backsheet
</commit_message>
<xml_diff>
--- a/Documentos/ACT-117C.xlsx
+++ b/Documentos/ACT-117C.xlsx
@@ -424,7 +424,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="201">
+  <cellXfs count="202">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -955,6 +955,9 @@
     </xf>
     <xf numFmtId="169" fontId="17" fillId="0" borderId="17" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -2256,7 +2259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q50"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.6640625" customWidth="1" min="1" max="1"/>
@@ -2527,7 +2530,6 @@
     <row r="15">
       <c r="H15" s="8" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="9" t="n">
         <v>17</v>
@@ -3958,48 +3960,48 @@
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="47" t="n"/>
       <c r="B23" s="130" t="n"/>
-      <c r="C23" s="65" t="n"/>
-      <c r="D23" s="131" t="n"/>
-      <c r="E23" s="131" t="n"/>
-      <c r="F23" s="131" t="n"/>
-      <c r="G23" s="131" t="n"/>
-      <c r="H23" s="131" t="n"/>
-      <c r="I23" s="131" t="n"/>
-      <c r="J23" s="131" t="n"/>
-      <c r="K23" s="131" t="n"/>
-      <c r="L23" s="131" t="n"/>
-      <c r="M23" s="131" t="n"/>
-      <c r="N23" s="131" t="n"/>
-      <c r="O23" s="131" t="n"/>
-      <c r="P23" s="131" t="n"/>
-      <c r="Q23" s="131" t="n"/>
-      <c r="R23" s="132" t="n"/>
+      <c r="C23" s="195" t="n"/>
+      <c r="D23" s="195" t="n"/>
+      <c r="E23" s="195" t="n"/>
+      <c r="F23" s="195" t="n"/>
+      <c r="G23" s="195" t="n"/>
+      <c r="H23" s="195" t="n"/>
+      <c r="I23" s="195" t="n"/>
+      <c r="J23" s="195" t="n"/>
+      <c r="K23" s="195" t="n"/>
+      <c r="L23" s="195" t="n"/>
+      <c r="M23" s="195" t="n"/>
+      <c r="N23" s="195" t="n"/>
+      <c r="O23" s="195" t="n"/>
+      <c r="P23" s="195" t="n"/>
+      <c r="Q23" s="195" t="n"/>
+      <c r="R23" s="195" t="n"/>
       <c r="S23" s="47" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="47" t="n"/>
-      <c r="B24" s="130" t="n"/>
-      <c r="C24" s="65" t="n"/>
-      <c r="D24" s="131" t="n"/>
-      <c r="E24" s="131" t="n"/>
-      <c r="F24" s="131" t="n"/>
-      <c r="G24" s="131" t="n"/>
-      <c r="H24" s="131" t="n"/>
-      <c r="I24" s="131" t="n"/>
-      <c r="J24" s="131" t="n"/>
-      <c r="K24" s="131" t="n"/>
-      <c r="L24" s="131" t="n"/>
-      <c r="M24" s="131" t="n"/>
-      <c r="N24" s="131" t="n"/>
-      <c r="O24" s="131" t="n"/>
-      <c r="P24" s="131" t="n"/>
-      <c r="Q24" s="131" t="n"/>
-      <c r="R24" s="132" t="n"/>
+      <c r="B24" s="201" t="n"/>
+      <c r="C24" s="195" t="n"/>
+      <c r="D24" s="195" t="n"/>
+      <c r="E24" s="195" t="n"/>
+      <c r="F24" s="195" t="n"/>
+      <c r="G24" s="195" t="n"/>
+      <c r="H24" s="195" t="n"/>
+      <c r="I24" s="195" t="n"/>
+      <c r="J24" s="195" t="n"/>
+      <c r="K24" s="195" t="n"/>
+      <c r="L24" s="195" t="n"/>
+      <c r="M24" s="195" t="n"/>
+      <c r="N24" s="195" t="n"/>
+      <c r="O24" s="195" t="n"/>
+      <c r="P24" s="195" t="n"/>
+      <c r="Q24" s="195" t="n"/>
+      <c r="R24" s="195" t="n"/>
       <c r="S24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="47" t="n"/>
-      <c r="B25" s="198" t="n"/>
+      <c r="B25" s="201" t="n"/>
       <c r="C25" s="195" t="n"/>
       <c r="D25" s="195" t="n"/>
       <c r="E25" s="195" t="n"/>
@@ -4015,12 +4017,12 @@
       <c r="O25" s="195" t="n"/>
       <c r="P25" s="195" t="n"/>
       <c r="Q25" s="195" t="n"/>
-      <c r="R25" s="196" t="n"/>
+      <c r="R25" s="195" t="n"/>
       <c r="S25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="47" t="n"/>
-      <c r="B26" s="194" t="n"/>
+      <c r="B26" s="201" t="n"/>
       <c r="C26" s="195" t="n"/>
       <c r="D26" s="195" t="n"/>
       <c r="E26" s="195" t="n"/>
@@ -4036,12 +4038,12 @@
       <c r="O26" s="195" t="n"/>
       <c r="P26" s="195" t="n"/>
       <c r="Q26" s="195" t="n"/>
-      <c r="R26" s="196" t="n"/>
+      <c r="R26" s="195" t="n"/>
       <c r="S26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="47" t="n"/>
-      <c r="B27" s="194" t="n"/>
+      <c r="B27" s="201" t="n"/>
       <c r="C27" s="195" t="n"/>
       <c r="D27" s="195" t="n"/>
       <c r="E27" s="195" t="n"/>
@@ -4057,12 +4059,12 @@
       <c r="O27" s="195" t="n"/>
       <c r="P27" s="195" t="n"/>
       <c r="Q27" s="195" t="n"/>
-      <c r="R27" s="196" t="n"/>
+      <c r="R27" s="195" t="n"/>
       <c r="S27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="47" t="n"/>
-      <c r="B28" s="194" t="n"/>
+      <c r="B28" s="201" t="n"/>
       <c r="C28" s="195" t="n"/>
       <c r="D28" s="195" t="n"/>
       <c r="E28" s="195" t="n"/>
@@ -4078,12 +4080,12 @@
       <c r="O28" s="195" t="n"/>
       <c r="P28" s="195" t="n"/>
       <c r="Q28" s="195" t="n"/>
-      <c r="R28" s="196" t="n"/>
+      <c r="R28" s="195" t="n"/>
       <c r="S28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="47" t="n"/>
-      <c r="B29" s="194" t="n"/>
+      <c r="B29" s="201" t="n"/>
       <c r="C29" s="195" t="n"/>
       <c r="D29" s="195" t="n"/>
       <c r="E29" s="195" t="n"/>
@@ -4099,12 +4101,12 @@
       <c r="O29" s="195" t="n"/>
       <c r="P29" s="195" t="n"/>
       <c r="Q29" s="195" t="n"/>
-      <c r="R29" s="196" t="n"/>
+      <c r="R29" s="195" t="n"/>
       <c r="S29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="47" t="n"/>
-      <c r="B30" s="199" t="n"/>
+      <c r="B30" s="201" t="n"/>
       <c r="C30" s="195" t="n"/>
       <c r="D30" s="195" t="n"/>
       <c r="E30" s="195" t="n"/>
@@ -4120,12 +4122,12 @@
       <c r="O30" s="195" t="n"/>
       <c r="P30" s="195" t="n"/>
       <c r="Q30" s="195" t="n"/>
-      <c r="R30" s="196" t="n"/>
+      <c r="R30" s="195" t="n"/>
       <c r="S30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="47" t="n"/>
-      <c r="B31" s="194" t="n"/>
+      <c r="B31" s="201" t="n"/>
       <c r="C31" s="195" t="n"/>
       <c r="D31" s="195" t="n"/>
       <c r="E31" s="195" t="n"/>
@@ -4141,12 +4143,12 @@
       <c r="O31" s="195" t="n"/>
       <c r="P31" s="195" t="n"/>
       <c r="Q31" s="195" t="n"/>
-      <c r="R31" s="196" t="n"/>
+      <c r="R31" s="195" t="n"/>
       <c r="S31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="47" t="n"/>
-      <c r="B32" s="194" t="n"/>
+      <c r="B32" s="201" t="n"/>
       <c r="C32" s="195" t="n"/>
       <c r="D32" s="195" t="n"/>
       <c r="E32" s="195" t="n"/>
@@ -4162,12 +4164,12 @@
       <c r="O32" s="195" t="n"/>
       <c r="P32" s="195" t="n"/>
       <c r="Q32" s="195" t="n"/>
-      <c r="R32" s="196" t="n"/>
+      <c r="R32" s="195" t="n"/>
       <c r="S32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="47" t="n"/>
-      <c r="B33" s="194" t="n"/>
+      <c r="B33" s="201" t="n"/>
       <c r="C33" s="195" t="n"/>
       <c r="D33" s="195" t="n"/>
       <c r="E33" s="195" t="n"/>
@@ -4183,12 +4185,12 @@
       <c r="O33" s="195" t="n"/>
       <c r="P33" s="195" t="n"/>
       <c r="Q33" s="195" t="n"/>
-      <c r="R33" s="196" t="n"/>
+      <c r="R33" s="195" t="n"/>
       <c r="S33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="47" t="n"/>
-      <c r="B34" s="200" t="n"/>
+      <c r="B34" s="201" t="n"/>
       <c r="C34" s="195" t="n"/>
       <c r="D34" s="195" t="n"/>
       <c r="E34" s="195" t="n"/>
@@ -4204,12 +4206,12 @@
       <c r="O34" s="195" t="n"/>
       <c r="P34" s="195" t="n"/>
       <c r="Q34" s="195" t="n"/>
-      <c r="R34" s="196" t="n"/>
+      <c r="R34" s="195" t="n"/>
       <c r="S34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="47" t="n"/>
-      <c r="B35" s="199" t="n"/>
+      <c r="B35" s="201" t="n"/>
       <c r="C35" s="195" t="n"/>
       <c r="D35" s="195" t="n"/>
       <c r="E35" s="195" t="n"/>
@@ -4225,7 +4227,7 @@
       <c r="O35" s="195" t="n"/>
       <c r="P35" s="195" t="n"/>
       <c r="Q35" s="195" t="n"/>
-      <c r="R35" s="196" t="n"/>
+      <c r="R35" s="195" t="n"/>
       <c r="S35" s="47" t="n"/>
     </row>
     <row r="36">
@@ -4630,27 +4632,22 @@
       <c r="S52" s="47" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="60">
-    <mergeCell ref="B32:R32"/>
+  <mergeCells count="50">
+    <mergeCell ref="B23:R35"/>
     <mergeCell ref="B4:R4"/>
-    <mergeCell ref="B26:R26"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B35:R35"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="N18:P18"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="B47:R47"/>
-    <mergeCell ref="B25:R25"/>
     <mergeCell ref="N8:P8"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B31:R31"/>
     <mergeCell ref="B46:R46"/>
     <mergeCell ref="B22:R22"/>
     <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B27:R27"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="B21:R21"/>
     <mergeCell ref="N10:P10"/>
@@ -4666,13 +4663,10 @@
     <mergeCell ref="B44:R44"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="G15:H15"/>
-    <mergeCell ref="B29:R29"/>
     <mergeCell ref="H7:I7"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B38:R38"/>
-    <mergeCell ref="B34:R34"/>
     <mergeCell ref="K18:M18"/>
-    <mergeCell ref="B28:R28"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="I14:J14"/>
@@ -4684,9 +4678,7 @@
     <mergeCell ref="K7:L7"/>
     <mergeCell ref="B40:R40"/>
     <mergeCell ref="J10:L10"/>
-    <mergeCell ref="B30:R30"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B33:R33"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="B45:R45"/>
     <mergeCell ref="B41:R41"/>

</xml_diff>